<commit_message>
feat: Add SCD41 CO2 sensor, new global variables, and fan speed automation, and include v2 PCB BOM files.
</commit_message>
<xml_diff>
--- a/EasyEDA-Pro/BOM_ESPHome Wohnraumlueftung v2_PCB_PCB_ESPHome-Wohnraumlueftung-v2_2026-01-20_2026-02-06.xlsx
+++ b/EasyEDA-Pro/BOM_ESPHome Wohnraumlueftung v2_PCB_PCB_ESPHome-Wohnraumlueftung-v2_2026-01-20_2026-02-06.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="562" uniqueCount="252">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="830" uniqueCount="319">
   <si>
     <t>No.</t>
   </si>
@@ -55,15 +55,36 @@
     <t>LCSC Price</t>
   </si>
   <si>
-    <t>Mounting Style</t>
-  </si>
-  <si>
     <t>Device</t>
   </si>
   <si>
     <t>Name</t>
   </si>
   <si>
+    <t>Description</t>
+  </si>
+  <si>
+    <t>JLCPCB Part Class</t>
+  </si>
+  <si>
+    <t>LCSC Part Name</t>
+  </si>
+  <si>
+    <t>Mounting Type</t>
+  </si>
+  <si>
+    <t>Noise</t>
+  </si>
+  <si>
+    <t>Power(Watts)</t>
+  </si>
+  <si>
+    <t>Voltage-Supply(Max)</t>
+  </si>
+  <si>
+    <t>Voltage Rating (Max)</t>
+  </si>
+  <si>
     <t>1</t>
   </si>
   <si>
@@ -91,13 +112,13 @@
     <t>LCSC</t>
   </si>
   <si>
-    <t>DIP</t>
+    <t>Extended Part</t>
   </si>
   <si>
     <t>2</t>
   </si>
   <si>
-    <t>10uF 50V 1206</t>
+    <t>10uF</t>
   </si>
   <si>
     <t>C2</t>
@@ -106,16 +127,25 @@
     <t>C1206</t>
   </si>
   <si>
-    <t>GRM31CR61H106MA12L</t>
-  </si>
-  <si>
-    <t>muRata(村田)</t>
-  </si>
-  <si>
-    <t>C882507</t>
-  </si>
-  <si>
-    <t>SMT</t>
+    <t>CL31B106KBHNNNE</t>
+  </si>
+  <si>
+    <t>SAMSUNG(三星)</t>
+  </si>
+  <si>
+    <t>C89632</t>
+  </si>
+  <si>
+    <t>Capacitors</t>
+  </si>
+  <si>
+    <t>Multilayer Ceramic Capacitors MLCC - SMD/SMT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Capacitance:10uF Tolerance:±10% Tolerance:±10% Voltage Rating:50V Temperature Coefficient:X7R </t>
+  </si>
+  <si>
+    <t>10uF ±10% 50V</t>
   </si>
   <si>
     <t>3</t>
@@ -139,6 +169,9 @@
     <t>C49678</t>
   </si>
   <si>
+    <t>Basic Part</t>
+  </si>
+  <si>
     <t>4</t>
   </si>
   <si>
@@ -157,12 +190,15 @@
     <t>C2977552</t>
   </si>
   <si>
-    <t>Capacitors</t>
-  </si>
-  <si>
     <t>Aluminum Electrolytic Capacitors - SMD</t>
   </si>
   <si>
+    <t>Capacitance:470uF Tolerance:±20% Tolerance:±20% Voltage Rating:16V Ripple Current:185mA@120Hz Diameter:6.3mm Height - Seated (Max):7.7mm Lifetime:2000hrs@105℃ Operating Temperature:-40℃~+105℃ Operating Temperature:-40℃~+105℃</t>
+  </si>
+  <si>
+    <t>470uF ±20% 16V</t>
+  </si>
+  <si>
     <t>5</t>
   </si>
   <si>
@@ -178,13 +214,13 @@
     <t>CL10A226MQ8NRNC</t>
   </si>
   <si>
-    <t>SAMSUNG(三星)</t>
-  </si>
-  <si>
     <t>C59461</t>
   </si>
   <si>
-    <t>Multilayer Ceramic Capacitors MLCC - SMD/SMT</t>
+    <t>Capacitance:22uF Tolerance:±20% Tolerance:±20% Voltage Rating:6.3V Temperature Coefficient:X5R</t>
+  </si>
+  <si>
+    <t>22uF ±20% 6.3V</t>
   </si>
   <si>
     <t>6</t>
@@ -205,12 +241,15 @@
     <t>C2918360</t>
   </si>
   <si>
+    <t>Capacitance:100uF Tolerance:±20% Tolerance:±20% Voltage Rating:25V Ripple Current:78mA@120Hz Equivalent Series Resistance(ESR):- Diameter:6.3mm Height - Seated (Max):5.4mm Lifetime:2000hrs@105℃ Operating Temperature:-40℃~+105℃ Operating Temperature:-40℃~+</t>
+  </si>
+  <si>
+    <t>100uF ±20% 25V</t>
+  </si>
+  <si>
     <t>7</t>
   </si>
   <si>
-    <t>10uF</t>
-  </si>
-  <si>
     <t>C28</t>
   </si>
   <si>
@@ -223,6 +262,12 @@
     <t>C39232</t>
   </si>
   <si>
+    <t>Capacitance:10uF Tolerance:±10% Tolerance:±10% Voltage Rating:25V Temperature Coefficient:X7R</t>
+  </si>
+  <si>
+    <t>10uF ±10% 25V</t>
+  </si>
+  <si>
     <t>8</t>
   </si>
   <si>
@@ -250,6 +295,12 @@
     <t>SS14_C6069588</t>
   </si>
   <si>
+    <t>Diode Configuration:Independent Voltage - Forward(Vf@If):550mV@1A Voltage - DC Reverse(Vr):40V Current - Rectified:1A Reverse Leakage Current (Ir):100uA@40V Operating Junction Temperature Range:-55℃~+150℃ Operating Junction Temperature Range:-55℃~+150℃ No</t>
+  </si>
+  <si>
+    <t>电压:40V 电流:1A</t>
+  </si>
+  <si>
     <t>9</t>
   </si>
   <si>
@@ -289,6 +340,18 @@
     <t>Pin Headers</t>
   </si>
   <si>
+    <t>Pin Structure:1x3P Pitch:2.54mm Circluar Pins/Square Pins:Pin Header Mounting Type:Through Hole Number of Rows:1 Number of Pins:3P Current Rating:3A Voltage Rating (Max):1kV Length of Mating Pin:6mm Insulation Height:2.5mm Length of End Connection Pin:3mm</t>
+  </si>
+  <si>
+    <t>1x3P 间距:2.54mm 方针 直插</t>
+  </si>
+  <si>
+    <t>Through Hole</t>
+  </si>
+  <si>
+    <t>1kV</t>
+  </si>
+  <si>
     <t>11</t>
   </si>
   <si>
@@ -307,6 +370,15 @@
     <t>C541879</t>
   </si>
   <si>
+    <t>Pin Structure:1x4P Pitch:1.27mm Row Spacing:- Circluar Pins/Square Pins:- Mounting Type:Through Hole Number of Rows:1 Number of Pins:4P Current Rating:- Voltage Rating (Max):- Length of Mating Pin:3.9mm Insulation Height:1mm Length of End Connection Pin:2</t>
+  </si>
+  <si>
+    <t>1x4P 间距:1.27mm 直插</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
     <t>12</t>
   </si>
   <si>
@@ -334,6 +406,12 @@
     <t>Power Inductors</t>
   </si>
   <si>
+    <t>Inductance:470uH Tolerance:±20% Tolerance:±20% Current Rating:500mA Current - Saturation(Isat):- DC Resistance(DCR):1.27Ω Type:- Ratings:-</t>
+  </si>
+  <si>
+    <t>470uH ±20%</t>
+  </si>
+  <si>
     <t>13</t>
   </si>
   <si>
@@ -355,6 +433,12 @@
     <t>C6808101</t>
   </si>
   <si>
+    <t>Inductance:3.9uH Tolerance:±20% Tolerance:±20% Current Rating:2.3A Current - Saturation(Isat):3.3A Type:Magnetic Shielded Inductor</t>
+  </si>
+  <si>
+    <t>3.9uH ±20% 3.3A 4x4x3mm</t>
+  </si>
+  <si>
     <t>14</t>
   </si>
   <si>
@@ -382,6 +466,12 @@
     <t>AO3401_C6575062</t>
   </si>
   <si>
+    <t>Number:1 P-Channel Drain to Source Voltage:30V Current - Continuous Drain(Id):4.1A RDS(on):65mΩ@4.5V,4A Pd - Power Dissipation:1.25W Gate Threshold Voltage (Vgs(th)):1.3V Input Capacitance(Ciss):870pF@0V Reverse Transfer Capacitance (Crss@Vds):10pF Operat</t>
+  </si>
+  <si>
+    <t>1个P沟道 耐压:30V 电流:4.1A</t>
+  </si>
+  <si>
     <t>15</t>
   </si>
   <si>
@@ -406,10 +496,16 @@
     <t>S8050_C20069125</t>
   </si>
   <si>
+    <t>type:NPN Current - Collector(Ic):500mA Collector - Emitter Voltage VCEO:25V Pd - Power Dissipation:300mW DC Current Gain:120@50mA,1.0V DC Current Gain:120@50mA,1.0V Transition frequency(fT):100MHz Current - Collector Cutoff:100nA Vce Saturation(VCE(sat)):</t>
+  </si>
+  <si>
+    <t>hFE:200-350，丝印:J3Y NPN 500mA 25V</t>
+  </si>
+  <si>
     <t>16</t>
   </si>
   <si>
-    <t>RES 4.7kΩ</t>
+    <t>4.7kΩ</t>
   </si>
   <si>
     <t>R1,R2</t>
@@ -418,19 +514,31 @@
     <t>R0603</t>
   </si>
   <si>
-    <t>PANASONIC(松下)</t>
-  </si>
-  <si>
-    <t>C336551</t>
-  </si>
-  <si>
-    <t>Sensors</t>
-  </si>
-  <si>
-    <t>NTC Thermistors</t>
-  </si>
-  <si>
-    <t>ERTJ1VT472J</t>
+    <t>0603WAF4701T5E</t>
+  </si>
+  <si>
+    <t>UNI-ROYAL(厚声)</t>
+  </si>
+  <si>
+    <t>C23162</t>
+  </si>
+  <si>
+    <t>Resistors</t>
+  </si>
+  <si>
+    <t>Chip Resistor - Surface Mount</t>
+  </si>
+  <si>
+    <t>Type:Thick Film Resistor Resistance:4.7kΩ Tolerance:±1% Tolerance:±1% Power(Watts):100mW Voltage-Supply(Max):75V Temperature Coefficient:±100ppm/℃ Temperature Coefficient:±100ppm/℃ Operating Temperature:-55℃~+155℃ Operating Temperature:-55℃~+155℃</t>
+  </si>
+  <si>
+    <t>4.7kΩ ±1% 100mW 厚膜电阻</t>
+  </si>
+  <si>
+    <t>100mW</t>
+  </si>
+  <si>
+    <t>75V</t>
   </si>
   <si>
     <t>17</t>
@@ -457,7 +565,7 @@
     <t>10kΩ</t>
   </si>
   <si>
-    <t>R4,R5,U24</t>
+    <t>R4,R5</t>
   </si>
   <si>
     <t>HoAR0603-1/10W-10KR-0.1%-TCR25</t>
@@ -478,15 +586,45 @@
     <t>0603WAF1002T5E</t>
   </si>
   <si>
-    <t>UNI-ROYAL(厚声)</t>
-  </si>
-  <si>
     <t>C25804</t>
   </si>
   <si>
     <t>20</t>
   </si>
   <si>
+    <t>2.2kΩ</t>
+  </si>
+  <si>
+    <t>R8</t>
+  </si>
+  <si>
+    <t>R0805</t>
+  </si>
+  <si>
+    <t>0805W8F2201T5E</t>
+  </si>
+  <si>
+    <t>C17520</t>
+  </si>
+  <si>
+    <t>0805W8F2201T5E_C17520</t>
+  </si>
+  <si>
+    <t>Type:Thick Film Resistor Resistance:2.2kΩ Tolerance:±1% Tolerance:±1% Power(Watts):125mW Voltage-Supply(Max):150V Temperature Coefficient:±100ppm/℃ Temperature Coefficient:±100ppm/℃ Operating Temperature:-55℃~+155℃ Operating Temperature:-55℃~+155℃</t>
+  </si>
+  <si>
+    <t>2.2kΩ ±1% 125mW 厚膜电阻</t>
+  </si>
+  <si>
+    <t>125mW</t>
+  </si>
+  <si>
+    <t>150V</t>
+  </si>
+  <si>
+    <t>21</t>
+  </si>
+  <si>
     <t>470Ω</t>
   </si>
   <si>
@@ -499,13 +637,13 @@
     <t>C23179</t>
   </si>
   <si>
-    <t>Resistors</t>
-  </si>
-  <si>
-    <t>Chip Resistor - Surface Mount</t>
-  </si>
-  <si>
-    <t>21</t>
+    <t>Type:Thick Film Resistor Resistance:470Ω Tolerance:±1% Tolerance:±1% Power(Watts):100mW Voltage-Supply(Max):75V Temperature Coefficient:±100ppm/℃ Temperature Coefficient:±100ppm/℃ Operating Temperature:-55℃~+155℃ Operating Temperature:-55℃~+155℃</t>
+  </si>
+  <si>
+    <t>470Ω ±1% 100mW 厚膜电阻</t>
+  </si>
+  <si>
+    <t>22</t>
   </si>
   <si>
     <t>RN1,RN2</t>
@@ -523,7 +661,16 @@
     <t>Resistor Networks, Arrays</t>
   </si>
   <si>
-    <t>22</t>
+    <t>Number of Resistors: Resistance:470Ω Tolerance:±5% Tolerance:±5% Power(Watts):62.5mW Temperature Coefficient:±200ppm/℃ Temperature Coefficient:±200ppm/℃ Number of Pins:</t>
+  </si>
+  <si>
+    <t>470Ω ±5%</t>
+  </si>
+  <si>
+    <t>62.5mW</t>
+  </si>
+  <si>
+    <t>23</t>
   </si>
   <si>
     <t>RN3</t>
@@ -535,7 +682,13 @@
     <t>C29718</t>
   </si>
   <si>
-    <t>23</t>
+    <t>Number of Resistors: Resistance:10kΩ Tolerance:±5% Tolerance:±5% Power(Watts): Temperature Coefficient:±200ppm/℃ Temperature Coefficient:±200ppm/℃ Number of Pins:</t>
+  </si>
+  <si>
+    <t>10kΩ ±5%</t>
+  </si>
+  <si>
+    <t>24</t>
   </si>
   <si>
     <t>TSR 1-2450_C6886877</t>
@@ -556,7 +709,7 @@
     <t>C6886877</t>
   </si>
   <si>
-    <t>24</t>
+    <t>25</t>
   </si>
   <si>
     <t>Screw Terminal 5.08 2P</t>
@@ -577,7 +730,7 @@
     <t>C474906</t>
   </si>
   <si>
-    <t>25</t>
+    <t>26</t>
   </si>
   <si>
     <t>TMPS10-112</t>
@@ -589,7 +742,7 @@
     <t>Traco Power</t>
   </si>
   <si>
-    <t>26</t>
+    <t>27</t>
   </si>
   <si>
     <t>PESD5V0S2BT_C5451656</t>
@@ -607,7 +760,7 @@
     <t>C5451656</t>
   </si>
   <si>
-    <t>27</t>
+    <t>28</t>
   </si>
   <si>
     <t>B254N02-0B7P51-H85C32</t>
@@ -628,7 +781,13 @@
     <t>Female Headers</t>
   </si>
   <si>
-    <t>28</t>
+    <t>Holes Structure:1x7P Pitch:2.54mm Circular Hole / Square Hole:Square Hole Mounting Type:Through Hole Number of Rows:1 Number of Positions:7P Current Rating:3A Holes Direction:Top Contact Material:Copper Alloy Operating Temperature:-40℃~+105℃ Operating Tem</t>
+  </si>
+  <si>
+    <t>1x7P 间距:2.54mm 直插</t>
+  </si>
+  <si>
+    <t>29</t>
   </si>
   <si>
     <t>FPC 0.5-14P LTH2.0</t>
@@ -649,7 +808,16 @@
     <t>FFC, FPC (Flat Flexible) Connector Assemblies</t>
   </si>
   <si>
-    <t>29</t>
+    <t>Locking Feature:Slide Lock Contact Type:Single-side Contact/Vertical Number of Contacts:14P Pitch:0.5mm Mounting Type:Surface Mount,Vertical FFC, FCB Thickness:0.3mm FFC, FCB Thickness:0.3mm Height Above Board:2mm Contact Material:Phosphor Bronze Contact</t>
+  </si>
+  <si>
+    <t>0.5-14P立贴正脚 编带</t>
+  </si>
+  <si>
+    <t>Surface Mount,Vertical</t>
+  </si>
+  <si>
+    <t>30</t>
   </si>
   <si>
     <t>PCA9685PW,118</t>
@@ -661,9 +829,6 @@
     <t>TSSOP-28_L9.7-W4.4-P0.65-LS6.4-TL</t>
   </si>
   <si>
-    <t>-</t>
-  </si>
-  <si>
     <t>NXP(恩智浦)</t>
   </si>
   <si>
@@ -673,7 +838,13 @@
     <t>LED Drivers</t>
   </si>
   <si>
-    <t>30</t>
+    <t>Type:- Voltage - Input(DC):2.3V~5.5V Voltage - Input(DC):2.3V~5.5V Frequency - Switching:100kHz~1MHz Frequency - Switching:100kHz~1MHz Number of Channels:16 Output Voltage:- Output Voltage:- Output Current:25mA Dimming:PWM Operating temperature:-40℃~+85℃</t>
+  </si>
+  <si>
+    <t>16通道、12位PWM Fm+ I2C总线LED控制器</t>
+  </si>
+  <si>
+    <t>31</t>
   </si>
   <si>
     <t>U27</t>
@@ -691,7 +862,16 @@
     <t>C2906861</t>
   </si>
   <si>
-    <t>31</t>
+    <t>Type:Thick Film Resistor Resistance:10kΩ Tolerance:±1% Tolerance:±1% Power(Watts):62.5mW Voltage-Supply(Max):50V Temperature Coefficient:±100ppm/℃ Temperature Coefficient:±100ppm/℃ Operating Temperature:-55℃~+155℃ Operating Temperature:-55℃~+155℃</t>
+  </si>
+  <si>
+    <t>10kΩ ±1% 62.5mW 厚膜电阻</t>
+  </si>
+  <si>
+    <t>50V</t>
+  </si>
+  <si>
+    <t>32</t>
   </si>
   <si>
     <t>KF128-2.54-2P</t>
@@ -709,7 +889,16 @@
     <t>Screw Terminal Blocks</t>
   </si>
   <si>
-    <t>32</t>
+    <t>Structure:1x2P Pitch:2.54mm Color:Green Mounting Style:Straight Current Rating (Max):8A Voltage Rating (Max):130V Number of Pins:2P Number of Rows:1 Wire Gauge - AWG:18~26 Wire Gauge - AWG:18~26 Wire Gauge - mm2:1 Wire Gauge - mm2:1 Number of PINs Per Row</t>
+  </si>
+  <si>
+    <t>2.54mm 1x2P 排数:1 每排P数:2 直插</t>
+  </si>
+  <si>
+    <t>130V</t>
+  </si>
+  <si>
+    <t>33</t>
   </si>
   <si>
     <t>KF128-2.54-4P</t>
@@ -724,7 +913,13 @@
     <t>C474922</t>
   </si>
   <si>
-    <t>33</t>
+    <t>Number of Positions or Pins:1x4P Pitch:2.54mm Color:Green Mounting Type:Through Hole Number of Pins:4P Number of Rows:1 Number of PINs Per Row:4 Current Rating:8A Voltage Rating (Max):130V Wire Gauge - AWG:18~26 Wire Gauge - mm2:1 Wire Gauge - mm2:1 Opera</t>
+  </si>
+  <si>
+    <t>1x4P 2.54mm 直插 排数:1 每排P数:4</t>
+  </si>
+  <si>
+    <t>34</t>
   </si>
   <si>
     <t>AP63203WU-7</t>
@@ -748,7 +943,13 @@
     <t>DC-DC Converters</t>
   </si>
   <si>
-    <t>34</t>
+    <t>Function:Buck Voltage - Supply:3.8V~32V Voltage - Supply:3.8V~32V Output Voltage:3.3V Output Voltage:3.3V Output Current:2A Frequency - Switching:1.1MHz Frequency - Switching:1.1MHz Operating Temperature:-40℃~+85℃@(TA) Operating Temperature:-40℃~+85℃@(TA)</t>
+  </si>
+  <si>
+    <t>3.8V至32V输入、2A低静态电流同步降压转换器，增强EMI抑制</t>
+  </si>
+  <si>
+    <t>35</t>
   </si>
   <si>
     <t>220pF@1kHz</t>
@@ -1143,13 +1344,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:Q36"/>
+  <dimension ref="A1:X37"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="17" width="20" customWidth="1"/>
+    <col min="1" max="24" width="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1201,1812 +1402,2621 @@
       <c r="Q1" t="s">
         <v>16</v>
       </c>
+      <c r="R1" t="s">
+        <v>17</v>
+      </c>
+      <c r="S1" t="s">
+        <v>18</v>
+      </c>
+      <c r="T1" t="s">
+        <v>19</v>
+      </c>
+      <c r="U1" t="s">
+        <v>20</v>
+      </c>
+      <c r="V1" t="s">
+        <v>21</v>
+      </c>
+      <c r="W1" t="s">
+        <v>22</v>
+      </c>
+      <c r="X1" t="s">
+        <v>23</v>
+      </c>
     </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="B2">
         <v>1</v>
       </c>
       <c r="C2" t="s">
-        <v>18</v>
+        <v>25</v>
       </c>
       <c r="D2" t="s">
-        <v>19</v>
+        <v>26</v>
       </c>
       <c r="E2" t="s">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="F2" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="G2" t="s">
-        <v>22</v>
+        <v>29</v>
       </c>
       <c r="H2" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="I2" t="s">
-        <v>24</v>
+        <v>31</v>
       </c>
       <c r="J2" t="s">
+        <v>32</v>
+      </c>
+      <c r="K2" t="s">
+        <v>28</v>
+      </c>
+      <c r="L2" t="s">
+        <v>28</v>
+      </c>
+      <c r="M2" t="s">
+        <v>28</v>
+      </c>
+      <c r="N2" t="s">
+        <v>28</v>
+      </c>
+      <c r="O2" t="s">
         <v>25</v>
       </c>
-      <c r="K2" t="s">
-        <v>21</v>
-      </c>
-      <c r="L2" t="s">
-        <v>21</v>
-      </c>
-      <c r="M2" t="s">
-        <v>21</v>
-      </c>
-      <c r="N2" t="s">
-        <v>21</v>
-      </c>
-      <c r="O2" t="s">
-        <v>26</v>
-      </c>
       <c r="P2" t="s">
-        <v>18</v>
+        <v>25</v>
       </c>
       <c r="Q2" t="s">
-        <v>18</v>
+        <v>28</v>
+      </c>
+      <c r="R2" t="s">
+        <v>33</v>
+      </c>
+      <c r="S2" t="s">
+        <v>28</v>
+      </c>
+      <c r="T2" t="s">
+        <v>28</v>
+      </c>
+      <c r="U2" t="s">
+        <v>28</v>
+      </c>
+      <c r="V2" t="s">
+        <v>28</v>
+      </c>
+      <c r="W2" t="s">
+        <v>28</v>
+      </c>
+      <c r="X2" t="s">
+        <v>28</v>
       </c>
     </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>27</v>
+        <v>34</v>
       </c>
       <c r="B3">
         <v>1</v>
       </c>
       <c r="C3" t="s">
-        <v>28</v>
+        <v>35</v>
       </c>
       <c r="D3" t="s">
-        <v>29</v>
+        <v>36</v>
       </c>
       <c r="E3" t="s">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="F3" t="s">
-        <v>21</v>
+        <v>35</v>
       </c>
       <c r="G3" t="s">
-        <v>31</v>
+        <v>38</v>
       </c>
       <c r="H3" t="s">
+        <v>39</v>
+      </c>
+      <c r="I3" t="s">
+        <v>40</v>
+      </c>
+      <c r="J3" t="s">
         <v>32</v>
       </c>
-      <c r="I3" t="s">
+      <c r="K3" t="s">
+        <v>41</v>
+      </c>
+      <c r="L3" t="s">
+        <v>42</v>
+      </c>
+      <c r="M3" t="s">
+        <v>28</v>
+      </c>
+      <c r="N3" t="s">
+        <v>28</v>
+      </c>
+      <c r="O3" t="s">
+        <v>38</v>
+      </c>
+      <c r="P3" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>43</v>
+      </c>
+      <c r="R3" t="s">
         <v>33</v>
       </c>
-      <c r="J3" t="s">
-        <v>25</v>
-      </c>
-      <c r="K3" t="s">
-        <v>21</v>
-      </c>
-      <c r="L3" t="s">
-        <v>21</v>
-      </c>
-      <c r="M3" t="s">
-        <v>21</v>
-      </c>
-      <c r="N3" t="s">
-        <v>21</v>
-      </c>
-      <c r="O3" t="s">
-        <v>34</v>
-      </c>
-      <c r="P3" t="s">
-        <v>28</v>
-      </c>
-      <c r="Q3" t="s">
+      <c r="S3" t="s">
+        <v>44</v>
+      </c>
+      <c r="T3" t="s">
+        <v>28</v>
+      </c>
+      <c r="U3" t="s">
+        <v>28</v>
+      </c>
+      <c r="V3" t="s">
+        <v>28</v>
+      </c>
+      <c r="W3" t="s">
+        <v>28</v>
+      </c>
+      <c r="X3" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="B4">
         <v>5</v>
       </c>
       <c r="C4" t="s">
-        <v>36</v>
+        <v>46</v>
       </c>
       <c r="D4" t="s">
-        <v>37</v>
+        <v>47</v>
       </c>
       <c r="E4" t="s">
-        <v>38</v>
+        <v>48</v>
       </c>
       <c r="F4" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="G4" t="s">
-        <v>39</v>
+        <v>49</v>
       </c>
       <c r="H4" t="s">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="I4" t="s">
-        <v>41</v>
+        <v>51</v>
       </c>
       <c r="J4" t="s">
-        <v>25</v>
+        <v>32</v>
       </c>
       <c r="K4" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="L4" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="M4" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="N4" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="O4" t="s">
-        <v>34</v>
+        <v>46</v>
       </c>
       <c r="P4" t="s">
-        <v>36</v>
+        <v>46</v>
       </c>
       <c r="Q4" t="s">
-        <v>36</v>
+        <v>28</v>
+      </c>
+      <c r="R4" t="s">
+        <v>52</v>
+      </c>
+      <c r="S4" t="s">
+        <v>28</v>
+      </c>
+      <c r="T4" t="s">
+        <v>28</v>
+      </c>
+      <c r="U4" t="s">
+        <v>28</v>
+      </c>
+      <c r="V4" t="s">
+        <v>28</v>
+      </c>
+      <c r="W4" t="s">
+        <v>28</v>
+      </c>
+      <c r="X4" t="s">
+        <v>28</v>
       </c>
     </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>42</v>
+        <v>53</v>
       </c>
       <c r="B5">
         <v>1</v>
       </c>
       <c r="C5" t="s">
-        <v>18</v>
+        <v>25</v>
       </c>
       <c r="D5" t="s">
-        <v>43</v>
+        <v>54</v>
       </c>
       <c r="E5" t="s">
-        <v>44</v>
+        <v>55</v>
       </c>
       <c r="F5" t="s">
-        <v>18</v>
+        <v>25</v>
       </c>
       <c r="G5" t="s">
-        <v>45</v>
+        <v>56</v>
       </c>
       <c r="H5" t="s">
-        <v>46</v>
+        <v>57</v>
       </c>
       <c r="I5" t="s">
-        <v>47</v>
+        <v>58</v>
       </c>
       <c r="J5" t="s">
+        <v>32</v>
+      </c>
+      <c r="K5" t="s">
+        <v>41</v>
+      </c>
+      <c r="L5" t="s">
+        <v>59</v>
+      </c>
+      <c r="M5" t="s">
+        <v>28</v>
+      </c>
+      <c r="N5" t="s">
+        <v>28</v>
+      </c>
+      <c r="O5" t="s">
+        <v>56</v>
+      </c>
+      <c r="P5" t="s">
         <v>25</v>
       </c>
-      <c r="K5" t="s">
-        <v>48</v>
-      </c>
-      <c r="L5" t="s">
-        <v>49</v>
-      </c>
-      <c r="M5" t="s">
-        <v>21</v>
-      </c>
-      <c r="N5" t="s">
-        <v>21</v>
-      </c>
-      <c r="O5" t="s">
-        <v>34</v>
-      </c>
-      <c r="P5" t="s">
-        <v>45</v>
-      </c>
       <c r="Q5" t="s">
-        <v>18</v>
+        <v>60</v>
+      </c>
+      <c r="R5" t="s">
+        <v>33</v>
+      </c>
+      <c r="S5" t="s">
+        <v>61</v>
+      </c>
+      <c r="T5" t="s">
+        <v>28</v>
+      </c>
+      <c r="U5" t="s">
+        <v>28</v>
+      </c>
+      <c r="V5" t="s">
+        <v>28</v>
+      </c>
+      <c r="W5" t="s">
+        <v>28</v>
+      </c>
+      <c r="X5" t="s">
+        <v>28</v>
       </c>
     </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>50</v>
+        <v>62</v>
       </c>
       <c r="B6">
         <v>2</v>
       </c>
       <c r="C6" t="s">
-        <v>51</v>
+        <v>63</v>
       </c>
       <c r="D6" t="s">
+        <v>64</v>
+      </c>
+      <c r="E6" t="s">
+        <v>65</v>
+      </c>
+      <c r="F6" t="s">
+        <v>63</v>
+      </c>
+      <c r="G6" t="s">
+        <v>66</v>
+      </c>
+      <c r="H6" t="s">
+        <v>39</v>
+      </c>
+      <c r="I6" t="s">
+        <v>67</v>
+      </c>
+      <c r="J6" t="s">
+        <v>32</v>
+      </c>
+      <c r="K6" t="s">
+        <v>41</v>
+      </c>
+      <c r="L6" t="s">
+        <v>42</v>
+      </c>
+      <c r="M6" t="s">
+        <v>28</v>
+      </c>
+      <c r="N6" t="s">
+        <v>28</v>
+      </c>
+      <c r="O6" t="s">
+        <v>66</v>
+      </c>
+      <c r="P6" t="s">
+        <v>63</v>
+      </c>
+      <c r="Q6" t="s">
+        <v>68</v>
+      </c>
+      <c r="R6" t="s">
         <v>52</v>
       </c>
-      <c r="E6" t="s">
-        <v>53</v>
-      </c>
-      <c r="F6" t="s">
-        <v>51</v>
-      </c>
-      <c r="G6" t="s">
-        <v>54</v>
-      </c>
-      <c r="H6" t="s">
-        <v>55</v>
-      </c>
-      <c r="I6" t="s">
-        <v>56</v>
-      </c>
-      <c r="J6" t="s">
-        <v>25</v>
-      </c>
-      <c r="K6" t="s">
-        <v>48</v>
-      </c>
-      <c r="L6" t="s">
-        <v>57</v>
-      </c>
-      <c r="M6" t="s">
-        <v>21</v>
-      </c>
-      <c r="N6" t="s">
-        <v>21</v>
-      </c>
-      <c r="O6" t="s">
-        <v>34</v>
-      </c>
-      <c r="P6" t="s">
-        <v>54</v>
-      </c>
-      <c r="Q6" t="s">
-        <v>51</v>
+      <c r="S6" t="s">
+        <v>69</v>
+      </c>
+      <c r="T6" t="s">
+        <v>28</v>
+      </c>
+      <c r="U6" t="s">
+        <v>28</v>
+      </c>
+      <c r="V6" t="s">
+        <v>28</v>
+      </c>
+      <c r="W6" t="s">
+        <v>28</v>
+      </c>
+      <c r="X6" t="s">
+        <v>28</v>
       </c>
     </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>58</v>
+        <v>70</v>
       </c>
       <c r="B7">
         <v>1</v>
       </c>
       <c r="C7" t="s">
+        <v>71</v>
+      </c>
+      <c r="D7" t="s">
+        <v>72</v>
+      </c>
+      <c r="E7" t="s">
+        <v>73</v>
+      </c>
+      <c r="F7" t="s">
+        <v>71</v>
+      </c>
+      <c r="G7" t="s">
+        <v>74</v>
+      </c>
+      <c r="H7" t="s">
+        <v>57</v>
+      </c>
+      <c r="I7" t="s">
+        <v>75</v>
+      </c>
+      <c r="J7" t="s">
+        <v>32</v>
+      </c>
+      <c r="K7" t="s">
+        <v>41</v>
+      </c>
+      <c r="L7" t="s">
         <v>59</v>
       </c>
-      <c r="D7" t="s">
-        <v>60</v>
-      </c>
-      <c r="E7" t="s">
-        <v>61</v>
-      </c>
-      <c r="F7" t="s">
-        <v>59</v>
-      </c>
-      <c r="G7" t="s">
-        <v>62</v>
-      </c>
-      <c r="H7" t="s">
-        <v>46</v>
-      </c>
-      <c r="I7" t="s">
-        <v>63</v>
-      </c>
-      <c r="J7" t="s">
-        <v>25</v>
-      </c>
-      <c r="K7" t="s">
-        <v>48</v>
-      </c>
-      <c r="L7" t="s">
-        <v>49</v>
-      </c>
       <c r="M7" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="N7" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="O7" t="s">
-        <v>34</v>
+        <v>74</v>
       </c>
       <c r="P7" t="s">
-        <v>62</v>
+        <v>71</v>
       </c>
       <c r="Q7" t="s">
-        <v>59</v>
+        <v>76</v>
+      </c>
+      <c r="R7" t="s">
+        <v>33</v>
+      </c>
+      <c r="S7" t="s">
+        <v>77</v>
+      </c>
+      <c r="T7" t="s">
+        <v>28</v>
+      </c>
+      <c r="U7" t="s">
+        <v>28</v>
+      </c>
+      <c r="V7" t="s">
+        <v>28</v>
+      </c>
+      <c r="W7" t="s">
+        <v>28</v>
+      </c>
+      <c r="X7" t="s">
+        <v>28</v>
       </c>
     </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>64</v>
+        <v>78</v>
       </c>
       <c r="B8">
         <v>1</v>
       </c>
       <c r="C8" t="s">
-        <v>65</v>
+        <v>35</v>
       </c>
       <c r="D8" t="s">
-        <v>66</v>
+        <v>79</v>
       </c>
       <c r="E8" t="s">
-        <v>67</v>
+        <v>80</v>
       </c>
       <c r="F8" t="s">
-        <v>65</v>
+        <v>35</v>
       </c>
       <c r="G8" t="s">
-        <v>68</v>
+        <v>81</v>
       </c>
       <c r="H8" t="s">
-        <v>55</v>
+        <v>39</v>
       </c>
       <c r="I8" t="s">
-        <v>69</v>
+        <v>82</v>
       </c>
       <c r="J8" t="s">
-        <v>25</v>
+        <v>32</v>
       </c>
       <c r="K8" t="s">
-        <v>48</v>
+        <v>41</v>
       </c>
       <c r="L8" t="s">
-        <v>57</v>
+        <v>42</v>
       </c>
       <c r="M8" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="N8" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="O8" t="s">
-        <v>34</v>
+        <v>81</v>
       </c>
       <c r="P8" t="s">
-        <v>68</v>
+        <v>35</v>
       </c>
       <c r="Q8" t="s">
-        <v>65</v>
+        <v>83</v>
+      </c>
+      <c r="R8" t="s">
+        <v>33</v>
+      </c>
+      <c r="S8" t="s">
+        <v>84</v>
+      </c>
+      <c r="T8" t="s">
+        <v>28</v>
+      </c>
+      <c r="U8" t="s">
+        <v>28</v>
+      </c>
+      <c r="V8" t="s">
+        <v>28</v>
+      </c>
+      <c r="W8" t="s">
+        <v>28</v>
+      </c>
+      <c r="X8" t="s">
+        <v>28</v>
       </c>
     </row>
-    <row r="9" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>70</v>
+        <v>85</v>
       </c>
       <c r="B9">
         <v>1</v>
       </c>
       <c r="C9" t="s">
-        <v>71</v>
+        <v>86</v>
       </c>
       <c r="D9" t="s">
-        <v>72</v>
+        <v>87</v>
       </c>
       <c r="E9" t="s">
-        <v>73</v>
+        <v>88</v>
       </c>
       <c r="F9" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="G9" t="s">
-        <v>71</v>
+        <v>86</v>
       </c>
       <c r="H9" t="s">
-        <v>74</v>
+        <v>89</v>
       </c>
       <c r="I9" t="s">
-        <v>75</v>
+        <v>90</v>
       </c>
       <c r="J9" t="s">
-        <v>25</v>
+        <v>32</v>
       </c>
       <c r="K9" t="s">
-        <v>76</v>
+        <v>91</v>
       </c>
       <c r="L9" t="s">
-        <v>77</v>
+        <v>92</v>
       </c>
       <c r="M9" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="N9" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="O9" t="s">
-        <v>34</v>
+        <v>93</v>
       </c>
       <c r="P9" t="s">
-        <v>78</v>
+        <v>86</v>
       </c>
       <c r="Q9" t="s">
-        <v>71</v>
+        <v>94</v>
+      </c>
+      <c r="R9" t="s">
+        <v>33</v>
+      </c>
+      <c r="S9" t="s">
+        <v>95</v>
+      </c>
+      <c r="T9" t="s">
+        <v>28</v>
+      </c>
+      <c r="U9" t="s">
+        <v>28</v>
+      </c>
+      <c r="V9" t="s">
+        <v>28</v>
+      </c>
+      <c r="W9" t="s">
+        <v>28</v>
+      </c>
+      <c r="X9" t="s">
+        <v>28</v>
       </c>
     </row>
-    <row r="10" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>79</v>
+        <v>96</v>
       </c>
       <c r="B10">
         <v>1</v>
       </c>
       <c r="C10" t="s">
-        <v>80</v>
+        <v>97</v>
       </c>
       <c r="D10" t="s">
-        <v>81</v>
+        <v>98</v>
       </c>
       <c r="E10" t="s">
-        <v>82</v>
+        <v>99</v>
       </c>
       <c r="F10" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="G10" t="s">
-        <v>80</v>
+        <v>97</v>
       </c>
       <c r="H10" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="I10" t="s">
-        <v>83</v>
+        <v>100</v>
       </c>
       <c r="J10" t="s">
-        <v>25</v>
+        <v>32</v>
       </c>
       <c r="K10" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="L10" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="M10" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="N10" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="O10" t="s">
-        <v>26</v>
+        <v>97</v>
       </c>
       <c r="P10" t="s">
-        <v>80</v>
+        <v>97</v>
       </c>
       <c r="Q10" t="s">
-        <v>80</v>
+        <v>28</v>
+      </c>
+      <c r="R10" t="s">
+        <v>33</v>
+      </c>
+      <c r="S10" t="s">
+        <v>97</v>
+      </c>
+      <c r="T10" t="s">
+        <v>28</v>
+      </c>
+      <c r="U10" t="s">
+        <v>28</v>
+      </c>
+      <c r="V10" t="s">
+        <v>28</v>
+      </c>
+      <c r="W10" t="s">
+        <v>28</v>
+      </c>
+      <c r="X10" t="s">
+        <v>28</v>
       </c>
     </row>
-    <row r="11" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>84</v>
+        <v>101</v>
       </c>
       <c r="B11">
         <v>1</v>
       </c>
       <c r="C11" t="s">
-        <v>85</v>
+        <v>102</v>
       </c>
       <c r="D11" t="s">
-        <v>86</v>
+        <v>103</v>
       </c>
       <c r="E11" t="s">
-        <v>87</v>
+        <v>104</v>
       </c>
       <c r="F11" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="G11" t="s">
-        <v>85</v>
+        <v>102</v>
       </c>
       <c r="H11" t="s">
-        <v>88</v>
+        <v>105</v>
       </c>
       <c r="I11" t="s">
-        <v>89</v>
+        <v>106</v>
       </c>
       <c r="J11" t="s">
-        <v>25</v>
+        <v>32</v>
       </c>
       <c r="K11" t="s">
-        <v>90</v>
+        <v>107</v>
       </c>
       <c r="L11" t="s">
-        <v>91</v>
+        <v>108</v>
       </c>
       <c r="M11" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="N11" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="O11" t="s">
-        <v>26</v>
+        <v>102</v>
       </c>
       <c r="P11" t="s">
-        <v>85</v>
+        <v>102</v>
       </c>
       <c r="Q11" t="s">
-        <v>85</v>
+        <v>109</v>
+      </c>
+      <c r="R11" t="s">
+        <v>33</v>
+      </c>
+      <c r="S11" t="s">
+        <v>110</v>
+      </c>
+      <c r="T11" t="s">
+        <v>111</v>
+      </c>
+      <c r="U11" t="s">
+        <v>28</v>
+      </c>
+      <c r="V11" t="s">
+        <v>28</v>
+      </c>
+      <c r="W11" t="s">
+        <v>28</v>
+      </c>
+      <c r="X11" t="s">
+        <v>112</v>
       </c>
     </row>
-    <row r="12" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>92</v>
+        <v>113</v>
       </c>
       <c r="B12">
         <v>1</v>
       </c>
       <c r="C12" t="s">
-        <v>93</v>
+        <v>114</v>
       </c>
       <c r="D12" t="s">
-        <v>94</v>
+        <v>115</v>
       </c>
       <c r="E12" t="s">
-        <v>95</v>
+        <v>116</v>
       </c>
       <c r="F12" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="G12" t="s">
-        <v>93</v>
+        <v>114</v>
       </c>
       <c r="H12" t="s">
-        <v>96</v>
+        <v>117</v>
       </c>
       <c r="I12" t="s">
-        <v>97</v>
+        <v>118</v>
       </c>
       <c r="J12" t="s">
-        <v>25</v>
+        <v>32</v>
       </c>
       <c r="K12" t="s">
-        <v>90</v>
+        <v>107</v>
       </c>
       <c r="L12" t="s">
-        <v>91</v>
+        <v>108</v>
       </c>
       <c r="M12" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="N12" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="O12" t="s">
-        <v>26</v>
+        <v>114</v>
       </c>
       <c r="P12" t="s">
-        <v>93</v>
+        <v>114</v>
       </c>
       <c r="Q12" t="s">
-        <v>93</v>
+        <v>119</v>
+      </c>
+      <c r="R12" t="s">
+        <v>33</v>
+      </c>
+      <c r="S12" t="s">
+        <v>120</v>
+      </c>
+      <c r="T12" t="s">
+        <v>111</v>
+      </c>
+      <c r="U12" t="s">
+        <v>28</v>
+      </c>
+      <c r="V12" t="s">
+        <v>28</v>
+      </c>
+      <c r="W12" t="s">
+        <v>28</v>
+      </c>
+      <c r="X12" t="s">
+        <v>121</v>
       </c>
     </row>
-    <row r="13" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>98</v>
+        <v>122</v>
       </c>
       <c r="B13">
         <v>1</v>
       </c>
       <c r="C13" t="s">
-        <v>99</v>
+        <v>123</v>
       </c>
       <c r="D13" t="s">
-        <v>100</v>
+        <v>124</v>
       </c>
       <c r="E13" t="s">
-        <v>101</v>
+        <v>125</v>
       </c>
       <c r="F13" t="s">
-        <v>99</v>
+        <v>123</v>
       </c>
       <c r="G13" t="s">
-        <v>102</v>
+        <v>126</v>
       </c>
       <c r="H13" t="s">
-        <v>103</v>
+        <v>127</v>
       </c>
       <c r="I13" t="s">
-        <v>104</v>
+        <v>128</v>
       </c>
       <c r="J13" t="s">
-        <v>25</v>
+        <v>32</v>
       </c>
       <c r="K13" t="s">
-        <v>105</v>
+        <v>129</v>
       </c>
       <c r="L13" t="s">
-        <v>106</v>
+        <v>130</v>
       </c>
       <c r="M13" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="N13" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="O13" t="s">
-        <v>34</v>
+        <v>126</v>
       </c>
       <c r="P13" t="s">
-        <v>102</v>
+        <v>123</v>
       </c>
       <c r="Q13" t="s">
-        <v>99</v>
+        <v>131</v>
+      </c>
+      <c r="R13" t="s">
+        <v>33</v>
+      </c>
+      <c r="S13" t="s">
+        <v>132</v>
+      </c>
+      <c r="T13" t="s">
+        <v>28</v>
+      </c>
+      <c r="U13" t="s">
+        <v>28</v>
+      </c>
+      <c r="V13" t="s">
+        <v>28</v>
+      </c>
+      <c r="W13" t="s">
+        <v>28</v>
+      </c>
+      <c r="X13" t="s">
+        <v>28</v>
       </c>
     </row>
-    <row r="14" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>107</v>
+        <v>133</v>
       </c>
       <c r="B14">
         <v>1</v>
       </c>
       <c r="C14" t="s">
-        <v>108</v>
+        <v>134</v>
       </c>
       <c r="D14" t="s">
-        <v>109</v>
+        <v>135</v>
       </c>
       <c r="E14" t="s">
-        <v>110</v>
+        <v>136</v>
       </c>
       <c r="F14" t="s">
-        <v>108</v>
+        <v>134</v>
       </c>
       <c r="G14" t="s">
-        <v>111</v>
+        <v>137</v>
       </c>
       <c r="H14" t="s">
-        <v>112</v>
+        <v>138</v>
       </c>
       <c r="I14" t="s">
-        <v>113</v>
+        <v>139</v>
       </c>
       <c r="J14" t="s">
-        <v>25</v>
+        <v>32</v>
       </c>
       <c r="K14" t="s">
-        <v>105</v>
+        <v>129</v>
       </c>
       <c r="L14" t="s">
-        <v>106</v>
+        <v>130</v>
       </c>
       <c r="M14" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="N14" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="O14" t="s">
-        <v>34</v>
+        <v>137</v>
       </c>
       <c r="P14" t="s">
-        <v>111</v>
+        <v>134</v>
       </c>
       <c r="Q14" t="s">
-        <v>108</v>
+        <v>140</v>
+      </c>
+      <c r="R14" t="s">
+        <v>33</v>
+      </c>
+      <c r="S14" t="s">
+        <v>141</v>
+      </c>
+      <c r="T14" t="s">
+        <v>28</v>
+      </c>
+      <c r="U14" t="s">
+        <v>28</v>
+      </c>
+      <c r="V14" t="s">
+        <v>28</v>
+      </c>
+      <c r="W14" t="s">
+        <v>28</v>
+      </c>
+      <c r="X14" t="s">
+        <v>28</v>
       </c>
     </row>
-    <row r="15" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>114</v>
+        <v>142</v>
       </c>
       <c r="B15">
         <v>1</v>
       </c>
       <c r="C15" t="s">
-        <v>115</v>
+        <v>143</v>
       </c>
       <c r="D15" t="s">
-        <v>116</v>
+        <v>144</v>
       </c>
       <c r="E15" t="s">
-        <v>117</v>
+        <v>145</v>
       </c>
       <c r="F15" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="G15" t="s">
-        <v>115</v>
+        <v>143</v>
       </c>
       <c r="H15" t="s">
-        <v>118</v>
+        <v>146</v>
       </c>
       <c r="I15" t="s">
-        <v>119</v>
+        <v>147</v>
       </c>
       <c r="J15" t="s">
-        <v>25</v>
+        <v>32</v>
       </c>
       <c r="K15" t="s">
-        <v>120</v>
+        <v>148</v>
       </c>
       <c r="L15" t="s">
-        <v>121</v>
+        <v>149</v>
       </c>
       <c r="M15" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="N15" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="O15" t="s">
-        <v>34</v>
+        <v>150</v>
       </c>
       <c r="P15" t="s">
-        <v>122</v>
+        <v>143</v>
       </c>
       <c r="Q15" t="s">
-        <v>115</v>
+        <v>151</v>
+      </c>
+      <c r="R15" t="s">
+        <v>33</v>
+      </c>
+      <c r="S15" t="s">
+        <v>152</v>
+      </c>
+      <c r="T15" t="s">
+        <v>28</v>
+      </c>
+      <c r="U15" t="s">
+        <v>28</v>
+      </c>
+      <c r="V15" t="s">
+        <v>28</v>
+      </c>
+      <c r="W15" t="s">
+        <v>28</v>
+      </c>
+      <c r="X15" t="s">
+        <v>28</v>
       </c>
     </row>
-    <row r="16" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>123</v>
+        <v>153</v>
       </c>
       <c r="B16">
         <v>1</v>
       </c>
       <c r="C16" t="s">
-        <v>124</v>
+        <v>154</v>
       </c>
       <c r="D16" t="s">
-        <v>125</v>
+        <v>155</v>
       </c>
       <c r="E16" t="s">
-        <v>126</v>
+        <v>156</v>
       </c>
       <c r="F16" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="G16" t="s">
-        <v>124</v>
+        <v>154</v>
       </c>
       <c r="H16" t="s">
-        <v>127</v>
+        <v>157</v>
       </c>
       <c r="I16" t="s">
-        <v>128</v>
+        <v>158</v>
       </c>
       <c r="J16" t="s">
-        <v>25</v>
+        <v>32</v>
       </c>
       <c r="K16" t="s">
-        <v>120</v>
+        <v>148</v>
       </c>
       <c r="L16" t="s">
-        <v>129</v>
+        <v>159</v>
       </c>
       <c r="M16" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="N16" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="O16" t="s">
-        <v>34</v>
+        <v>160</v>
       </c>
       <c r="P16" t="s">
-        <v>130</v>
+        <v>154</v>
       </c>
       <c r="Q16" t="s">
-        <v>124</v>
+        <v>161</v>
+      </c>
+      <c r="R16" t="s">
+        <v>33</v>
+      </c>
+      <c r="S16" t="s">
+        <v>162</v>
+      </c>
+      <c r="T16" t="s">
+        <v>28</v>
+      </c>
+      <c r="U16" t="s">
+        <v>28</v>
+      </c>
+      <c r="V16" t="s">
+        <v>28</v>
+      </c>
+      <c r="W16" t="s">
+        <v>28</v>
+      </c>
+      <c r="X16" t="s">
+        <v>28</v>
       </c>
     </row>
-    <row r="17" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>131</v>
+        <v>163</v>
       </c>
       <c r="B17">
         <v>2</v>
       </c>
       <c r="C17" t="s">
-        <v>132</v>
+        <v>164</v>
       </c>
       <c r="D17" t="s">
-        <v>133</v>
+        <v>165</v>
       </c>
       <c r="E17" t="s">
-        <v>134</v>
+        <v>166</v>
       </c>
       <c r="F17" t="s">
-        <v>21</v>
+        <v>164</v>
       </c>
       <c r="G17" t="s">
-        <v>132</v>
+        <v>167</v>
       </c>
       <c r="H17" t="s">
-        <v>135</v>
+        <v>168</v>
       </c>
       <c r="I17" t="s">
-        <v>136</v>
+        <v>169</v>
       </c>
       <c r="J17" t="s">
-        <v>25</v>
+        <v>32</v>
       </c>
       <c r="K17" t="s">
-        <v>137</v>
+        <v>170</v>
       </c>
       <c r="L17" t="s">
-        <v>138</v>
+        <v>171</v>
       </c>
       <c r="M17" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="N17" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="O17" t="s">
-        <v>34</v>
+        <v>167</v>
       </c>
       <c r="P17" t="s">
-        <v>139</v>
+        <v>164</v>
       </c>
       <c r="Q17" t="s">
-        <v>132</v>
+        <v>172</v>
+      </c>
+      <c r="R17" t="s">
+        <v>52</v>
+      </c>
+      <c r="S17" t="s">
+        <v>173</v>
+      </c>
+      <c r="T17" t="s">
+        <v>28</v>
+      </c>
+      <c r="U17" t="s">
+        <v>28</v>
+      </c>
+      <c r="V17" t="s">
+        <v>174</v>
+      </c>
+      <c r="W17" t="s">
+        <v>175</v>
+      </c>
+      <c r="X17" t="s">
+        <v>28</v>
       </c>
     </row>
-    <row r="18" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>140</v>
+        <v>176</v>
       </c>
       <c r="B18">
         <v>1</v>
       </c>
       <c r="C18" t="s">
-        <v>141</v>
+        <v>177</v>
       </c>
       <c r="D18" t="s">
-        <v>142</v>
+        <v>178</v>
       </c>
       <c r="E18" t="s">
-        <v>134</v>
+        <v>166</v>
       </c>
       <c r="F18" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="G18" t="s">
-        <v>143</v>
+        <v>179</v>
       </c>
       <c r="H18" t="s">
-        <v>144</v>
+        <v>180</v>
       </c>
       <c r="I18" t="s">
-        <v>145</v>
+        <v>181</v>
       </c>
       <c r="J18" t="s">
-        <v>25</v>
+        <v>32</v>
       </c>
       <c r="K18" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="L18" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="M18" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="N18" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="O18" t="s">
-        <v>34</v>
+        <v>177</v>
       </c>
       <c r="P18" t="s">
-        <v>141</v>
+        <v>177</v>
       </c>
       <c r="Q18" t="s">
-        <v>141</v>
+        <v>28</v>
+      </c>
+      <c r="R18" t="s">
+        <v>33</v>
+      </c>
+      <c r="S18" t="s">
+        <v>28</v>
+      </c>
+      <c r="T18" t="s">
+        <v>28</v>
+      </c>
+      <c r="U18" t="s">
+        <v>28</v>
+      </c>
+      <c r="V18" t="s">
+        <v>28</v>
+      </c>
+      <c r="W18" t="s">
+        <v>28</v>
+      </c>
+      <c r="X18" t="s">
+        <v>28</v>
       </c>
     </row>
-    <row r="19" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>146</v>
+        <v>182</v>
       </c>
       <c r="B19">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C19" t="s">
-        <v>147</v>
+        <v>183</v>
       </c>
       <c r="D19" t="s">
-        <v>148</v>
+        <v>184</v>
       </c>
       <c r="E19" t="s">
-        <v>134</v>
+        <v>166</v>
       </c>
       <c r="F19" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="G19" t="s">
-        <v>149</v>
+        <v>185</v>
       </c>
       <c r="H19" t="s">
-        <v>150</v>
+        <v>186</v>
       </c>
       <c r="I19" t="s">
-        <v>151</v>
+        <v>187</v>
       </c>
       <c r="J19" t="s">
-        <v>25</v>
+        <v>32</v>
       </c>
       <c r="K19" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="L19" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="M19" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="N19" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="O19" t="s">
-        <v>34</v>
+        <v>183</v>
       </c>
       <c r="P19" t="s">
-        <v>147</v>
+        <v>183</v>
       </c>
       <c r="Q19" t="s">
-        <v>147</v>
+        <v>28</v>
+      </c>
+      <c r="R19" t="s">
+        <v>28</v>
+      </c>
+      <c r="S19" t="s">
+        <v>28</v>
+      </c>
+      <c r="T19" t="s">
+        <v>28</v>
+      </c>
+      <c r="U19" t="s">
+        <v>28</v>
+      </c>
+      <c r="V19" t="s">
+        <v>28</v>
+      </c>
+      <c r="W19" t="s">
+        <v>28</v>
+      </c>
+      <c r="X19" t="s">
+        <v>28</v>
       </c>
     </row>
-    <row r="20" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>152</v>
+        <v>188</v>
       </c>
       <c r="B20">
         <v>1</v>
       </c>
       <c r="C20" t="s">
-        <v>147</v>
+        <v>183</v>
       </c>
       <c r="D20" t="s">
-        <v>153</v>
+        <v>189</v>
       </c>
       <c r="E20" t="s">
-        <v>134</v>
+        <v>166</v>
       </c>
       <c r="F20" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="G20" t="s">
-        <v>154</v>
+        <v>190</v>
       </c>
       <c r="H20" t="s">
-        <v>155</v>
+        <v>168</v>
       </c>
       <c r="I20" t="s">
-        <v>156</v>
+        <v>191</v>
       </c>
       <c r="J20" t="s">
-        <v>25</v>
+        <v>32</v>
       </c>
       <c r="K20" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="L20" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="M20" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="N20" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="O20" t="s">
-        <v>34</v>
+        <v>183</v>
       </c>
       <c r="P20" t="s">
-        <v>147</v>
+        <v>183</v>
       </c>
       <c r="Q20" t="s">
-        <v>147</v>
+        <v>28</v>
+      </c>
+      <c r="R20" t="s">
+        <v>52</v>
+      </c>
+      <c r="S20" t="s">
+        <v>28</v>
+      </c>
+      <c r="T20" t="s">
+        <v>28</v>
+      </c>
+      <c r="U20" t="s">
+        <v>28</v>
+      </c>
+      <c r="V20" t="s">
+        <v>28</v>
+      </c>
+      <c r="W20" t="s">
+        <v>28</v>
+      </c>
+      <c r="X20" t="s">
+        <v>28</v>
       </c>
     </row>
-    <row r="21" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>157</v>
+        <v>192</v>
       </c>
       <c r="B21">
         <v>1</v>
       </c>
       <c r="C21" t="s">
-        <v>158</v>
+        <v>193</v>
       </c>
       <c r="D21" t="s">
-        <v>159</v>
+        <v>194</v>
       </c>
       <c r="E21" t="s">
-        <v>134</v>
+        <v>195</v>
       </c>
       <c r="F21" t="s">
-        <v>158</v>
+        <v>193</v>
       </c>
       <c r="G21" t="s">
-        <v>160</v>
+        <v>196</v>
       </c>
       <c r="H21" t="s">
-        <v>155</v>
+        <v>168</v>
       </c>
       <c r="I21" t="s">
-        <v>161</v>
+        <v>197</v>
       </c>
       <c r="J21" t="s">
-        <v>25</v>
+        <v>32</v>
       </c>
       <c r="K21" t="s">
-        <v>162</v>
+        <v>170</v>
       </c>
       <c r="L21" t="s">
-        <v>163</v>
+        <v>171</v>
       </c>
       <c r="M21" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="N21" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="O21" t="s">
-        <v>34</v>
+        <v>198</v>
       </c>
       <c r="P21" t="s">
-        <v>160</v>
+        <v>193</v>
       </c>
       <c r="Q21" t="s">
-        <v>158</v>
+        <v>199</v>
+      </c>
+      <c r="R21" t="s">
+        <v>52</v>
+      </c>
+      <c r="S21" t="s">
+        <v>200</v>
+      </c>
+      <c r="T21" t="s">
+        <v>28</v>
+      </c>
+      <c r="U21" t="s">
+        <v>28</v>
+      </c>
+      <c r="V21" t="s">
+        <v>201</v>
+      </c>
+      <c r="W21" t="s">
+        <v>202</v>
+      </c>
+      <c r="X21" t="s">
+        <v>28</v>
       </c>
     </row>
-    <row r="22" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>164</v>
+        <v>203</v>
       </c>
       <c r="B22">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C22" t="s">
-        <v>158</v>
+        <v>204</v>
       </c>
       <c r="D22" t="s">
-        <v>165</v>
+        <v>205</v>
       </c>
       <c r="E22" t="s">
         <v>166</v>
       </c>
       <c r="F22" t="s">
-        <v>158</v>
+        <v>204</v>
       </c>
       <c r="G22" t="s">
-        <v>167</v>
+        <v>206</v>
       </c>
       <c r="H22" t="s">
-        <v>155</v>
+        <v>168</v>
       </c>
       <c r="I22" t="s">
+        <v>207</v>
+      </c>
+      <c r="J22" t="s">
+        <v>32</v>
+      </c>
+      <c r="K22" t="s">
+        <v>170</v>
+      </c>
+      <c r="L22" t="s">
+        <v>171</v>
+      </c>
+      <c r="M22" t="s">
+        <v>28</v>
+      </c>
+      <c r="N22" t="s">
+        <v>28</v>
+      </c>
+      <c r="O22" t="s">
+        <v>206</v>
+      </c>
+      <c r="P22" t="s">
+        <v>204</v>
+      </c>
+      <c r="Q22" t="s">
+        <v>208</v>
+      </c>
+      <c r="R22" t="s">
+        <v>52</v>
+      </c>
+      <c r="S22" t="s">
+        <v>209</v>
+      </c>
+      <c r="T22" t="s">
+        <v>28</v>
+      </c>
+      <c r="U22" t="s">
+        <v>28</v>
+      </c>
+      <c r="V22" t="s">
+        <v>174</v>
+      </c>
+      <c r="W22" t="s">
+        <v>175</v>
+      </c>
+      <c r="X22" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="23" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>210</v>
+      </c>
+      <c r="B23">
+        <v>2</v>
+      </c>
+      <c r="C23" t="s">
+        <v>204</v>
+      </c>
+      <c r="D23" t="s">
+        <v>211</v>
+      </c>
+      <c r="E23" t="s">
+        <v>212</v>
+      </c>
+      <c r="F23" t="s">
+        <v>204</v>
+      </c>
+      <c r="G23" t="s">
+        <v>213</v>
+      </c>
+      <c r="H23" t="s">
         <v>168</v>
       </c>
-      <c r="J22" t="s">
-        <v>25</v>
-      </c>
-      <c r="K22" t="s">
-        <v>162</v>
-      </c>
-      <c r="L22" t="s">
-        <v>169</v>
-      </c>
-      <c r="M22" t="s">
-        <v>21</v>
-      </c>
-      <c r="N22" t="s">
-        <v>21</v>
-      </c>
-      <c r="O22" t="s">
-        <v>34</v>
-      </c>
-      <c r="P22" t="s">
-        <v>167</v>
-      </c>
-      <c r="Q22" t="s">
-        <v>158</v>
+      <c r="I23" t="s">
+        <v>214</v>
+      </c>
+      <c r="J23" t="s">
+        <v>32</v>
+      </c>
+      <c r="K23" t="s">
+        <v>170</v>
+      </c>
+      <c r="L23" t="s">
+        <v>215</v>
+      </c>
+      <c r="M23" t="s">
+        <v>28</v>
+      </c>
+      <c r="N23" t="s">
+        <v>28</v>
+      </c>
+      <c r="O23" t="s">
+        <v>213</v>
+      </c>
+      <c r="P23" t="s">
+        <v>204</v>
+      </c>
+      <c r="Q23" t="s">
+        <v>216</v>
+      </c>
+      <c r="R23" t="s">
+        <v>33</v>
+      </c>
+      <c r="S23" t="s">
+        <v>217</v>
+      </c>
+      <c r="T23" t="s">
+        <v>28</v>
+      </c>
+      <c r="U23" t="s">
+        <v>28</v>
+      </c>
+      <c r="V23" t="s">
+        <v>218</v>
+      </c>
+      <c r="W23" t="s">
+        <v>28</v>
+      </c>
+      <c r="X23" t="s">
+        <v>28</v>
       </c>
     </row>
-    <row r="23" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
-        <v>170</v>
-      </c>
-      <c r="B23">
-        <v>1</v>
-      </c>
-      <c r="C23" t="s">
-        <v>147</v>
-      </c>
-      <c r="D23" t="s">
-        <v>171</v>
-      </c>
-      <c r="E23" t="s">
-        <v>166</v>
-      </c>
-      <c r="F23" t="s">
-        <v>147</v>
-      </c>
-      <c r="G23" t="s">
-        <v>172</v>
-      </c>
-      <c r="H23" t="s">
-        <v>155</v>
-      </c>
-      <c r="I23" t="s">
-        <v>173</v>
-      </c>
-      <c r="J23" t="s">
-        <v>25</v>
-      </c>
-      <c r="K23" t="s">
-        <v>162</v>
-      </c>
-      <c r="L23" t="s">
-        <v>169</v>
-      </c>
-      <c r="M23" t="s">
-        <v>21</v>
-      </c>
-      <c r="N23" t="s">
-        <v>21</v>
-      </c>
-      <c r="O23" t="s">
-        <v>34</v>
-      </c>
-      <c r="P23" t="s">
-        <v>172</v>
-      </c>
-      <c r="Q23" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="24" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>174</v>
+        <v>219</v>
       </c>
       <c r="B24">
         <v>1</v>
       </c>
       <c r="C24" t="s">
-        <v>175</v>
+        <v>183</v>
       </c>
       <c r="D24" t="s">
-        <v>176</v>
+        <v>220</v>
       </c>
       <c r="E24" t="s">
-        <v>177</v>
+        <v>212</v>
       </c>
       <c r="F24" t="s">
-        <v>21</v>
+        <v>183</v>
       </c>
       <c r="G24" t="s">
-        <v>178</v>
+        <v>221</v>
       </c>
       <c r="H24" t="s">
-        <v>179</v>
+        <v>168</v>
       </c>
       <c r="I24" t="s">
-        <v>180</v>
+        <v>222</v>
       </c>
       <c r="J24" t="s">
-        <v>25</v>
+        <v>32</v>
       </c>
       <c r="K24" t="s">
-        <v>21</v>
+        <v>170</v>
       </c>
       <c r="L24" t="s">
-        <v>21</v>
+        <v>215</v>
       </c>
       <c r="M24" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="N24" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="O24" t="s">
-        <v>26</v>
+        <v>221</v>
       </c>
       <c r="P24" t="s">
-        <v>175</v>
+        <v>183</v>
       </c>
       <c r="Q24" t="s">
-        <v>175</v>
+        <v>223</v>
+      </c>
+      <c r="R24" t="s">
+        <v>52</v>
+      </c>
+      <c r="S24" t="s">
+        <v>224</v>
+      </c>
+      <c r="T24" t="s">
+        <v>28</v>
+      </c>
+      <c r="U24" t="s">
+        <v>28</v>
+      </c>
+      <c r="V24" t="s">
+        <v>28</v>
+      </c>
+      <c r="W24" t="s">
+        <v>28</v>
+      </c>
+      <c r="X24" t="s">
+        <v>28</v>
       </c>
     </row>
-    <row r="25" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>181</v>
+        <v>225</v>
       </c>
       <c r="B25">
         <v>1</v>
       </c>
       <c r="C25" t="s">
-        <v>182</v>
+        <v>226</v>
       </c>
       <c r="D25" t="s">
-        <v>183</v>
+        <v>227</v>
       </c>
       <c r="E25" t="s">
-        <v>184</v>
+        <v>228</v>
       </c>
       <c r="F25" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="G25" t="s">
-        <v>185</v>
+        <v>229</v>
       </c>
       <c r="H25" t="s">
-        <v>186</v>
+        <v>230</v>
       </c>
       <c r="I25" t="s">
-        <v>187</v>
+        <v>231</v>
       </c>
       <c r="J25" t="s">
-        <v>25</v>
+        <v>32</v>
       </c>
       <c r="K25" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="L25" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="M25" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="N25" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="O25" t="s">
-        <v>26</v>
+        <v>226</v>
       </c>
       <c r="P25" t="s">
-        <v>182</v>
+        <v>226</v>
       </c>
       <c r="Q25" t="s">
-        <v>182</v>
+        <v>28</v>
+      </c>
+      <c r="R25" t="s">
+        <v>33</v>
+      </c>
+      <c r="S25" t="s">
+        <v>28</v>
+      </c>
+      <c r="T25" t="s">
+        <v>28</v>
+      </c>
+      <c r="U25" t="s">
+        <v>28</v>
+      </c>
+      <c r="V25" t="s">
+        <v>28</v>
+      </c>
+      <c r="W25" t="s">
+        <v>28</v>
+      </c>
+      <c r="X25" t="s">
+        <v>28</v>
       </c>
     </row>
-    <row r="26" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>188</v>
+        <v>232</v>
       </c>
       <c r="B26">
         <v>1</v>
       </c>
       <c r="C26" t="s">
-        <v>189</v>
+        <v>233</v>
       </c>
       <c r="D26" t="s">
-        <v>190</v>
+        <v>234</v>
       </c>
       <c r="E26" t="s">
-        <v>189</v>
+        <v>235</v>
       </c>
       <c r="F26" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="G26" t="s">
-        <v>21</v>
+        <v>236</v>
       </c>
       <c r="H26" t="s">
-        <v>21</v>
+        <v>237</v>
       </c>
       <c r="I26" t="s">
-        <v>21</v>
+        <v>238</v>
       </c>
       <c r="J26" t="s">
-        <v>191</v>
+        <v>32</v>
       </c>
       <c r="K26" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="L26" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="M26" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="N26" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="O26" t="s">
-        <v>26</v>
+        <v>233</v>
       </c>
       <c r="P26" t="s">
-        <v>189</v>
+        <v>233</v>
       </c>
       <c r="Q26" t="s">
-        <v>189</v>
+        <v>28</v>
+      </c>
+      <c r="R26" t="s">
+        <v>33</v>
+      </c>
+      <c r="S26" t="s">
+        <v>28</v>
+      </c>
+      <c r="T26" t="s">
+        <v>28</v>
+      </c>
+      <c r="U26" t="s">
+        <v>28</v>
+      </c>
+      <c r="V26" t="s">
+        <v>28</v>
+      </c>
+      <c r="W26" t="s">
+        <v>28</v>
+      </c>
+      <c r="X26" t="s">
+        <v>28</v>
       </c>
     </row>
-    <row r="27" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>192</v>
+        <v>239</v>
       </c>
       <c r="B27">
+        <v>1</v>
+      </c>
+      <c r="C27" t="s">
+        <v>240</v>
+      </c>
+      <c r="D27" t="s">
+        <v>241</v>
+      </c>
+      <c r="E27" t="s">
+        <v>240</v>
+      </c>
+      <c r="F27" t="s">
+        <v>28</v>
+      </c>
+      <c r="G27" t="s">
+        <v>28</v>
+      </c>
+      <c r="H27" t="s">
+        <v>28</v>
+      </c>
+      <c r="I27" t="s">
+        <v>28</v>
+      </c>
+      <c r="J27" t="s">
+        <v>242</v>
+      </c>
+      <c r="K27" t="s">
+        <v>28</v>
+      </c>
+      <c r="L27" t="s">
+        <v>28</v>
+      </c>
+      <c r="M27" t="s">
+        <v>28</v>
+      </c>
+      <c r="N27" t="s">
+        <v>28</v>
+      </c>
+      <c r="O27" t="s">
+        <v>240</v>
+      </c>
+      <c r="P27" t="s">
+        <v>240</v>
+      </c>
+      <c r="Q27" t="s">
+        <v>28</v>
+      </c>
+      <c r="R27" t="s">
+        <v>28</v>
+      </c>
+      <c r="S27" t="s">
+        <v>28</v>
+      </c>
+      <c r="T27" t="s">
+        <v>28</v>
+      </c>
+      <c r="U27" t="s">
+        <v>28</v>
+      </c>
+      <c r="V27" t="s">
+        <v>28</v>
+      </c>
+      <c r="W27" t="s">
+        <v>28</v>
+      </c>
+      <c r="X27" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="28" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>243</v>
+      </c>
+      <c r="B28">
         <v>10</v>
       </c>
-      <c r="C27" t="s">
-        <v>193</v>
-      </c>
-      <c r="D27" t="s">
-        <v>194</v>
-      </c>
-      <c r="E27" t="s">
-        <v>117</v>
-      </c>
-      <c r="F27" t="s">
-        <v>21</v>
-      </c>
-      <c r="G27" t="s">
-        <v>195</v>
-      </c>
-      <c r="H27" t="s">
-        <v>196</v>
-      </c>
-      <c r="I27" t="s">
-        <v>197</v>
-      </c>
-      <c r="J27" t="s">
-        <v>25</v>
-      </c>
-      <c r="K27" t="s">
-        <v>21</v>
-      </c>
-      <c r="L27" t="s">
-        <v>21</v>
-      </c>
-      <c r="M27" t="s">
-        <v>21</v>
-      </c>
-      <c r="N27" t="s">
-        <v>21</v>
-      </c>
-      <c r="O27" t="s">
-        <v>34</v>
-      </c>
-      <c r="P27" t="s">
-        <v>193</v>
-      </c>
-      <c r="Q27" t="s">
-        <v>193</v>
+      <c r="C28" t="s">
+        <v>244</v>
+      </c>
+      <c r="D28" t="s">
+        <v>245</v>
+      </c>
+      <c r="E28" t="s">
+        <v>145</v>
+      </c>
+      <c r="F28" t="s">
+        <v>28</v>
+      </c>
+      <c r="G28" t="s">
+        <v>246</v>
+      </c>
+      <c r="H28" t="s">
+        <v>247</v>
+      </c>
+      <c r="I28" t="s">
+        <v>248</v>
+      </c>
+      <c r="J28" t="s">
+        <v>32</v>
+      </c>
+      <c r="K28" t="s">
+        <v>28</v>
+      </c>
+      <c r="L28" t="s">
+        <v>28</v>
+      </c>
+      <c r="M28" t="s">
+        <v>28</v>
+      </c>
+      <c r="N28" t="s">
+        <v>28</v>
+      </c>
+      <c r="O28" t="s">
+        <v>244</v>
+      </c>
+      <c r="P28" t="s">
+        <v>244</v>
+      </c>
+      <c r="Q28" t="s">
+        <v>28</v>
+      </c>
+      <c r="R28" t="s">
+        <v>33</v>
+      </c>
+      <c r="S28" t="s">
+        <v>28</v>
+      </c>
+      <c r="T28" t="s">
+        <v>28</v>
+      </c>
+      <c r="U28" t="s">
+        <v>28</v>
+      </c>
+      <c r="V28" t="s">
+        <v>28</v>
+      </c>
+      <c r="W28" t="s">
+        <v>28</v>
+      </c>
+      <c r="X28" t="s">
+        <v>28</v>
       </c>
     </row>
-    <row r="28" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
-        <v>198</v>
-      </c>
-      <c r="B28">
+    <row r="29" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>249</v>
+      </c>
+      <c r="B29">
         <v>2</v>
       </c>
-      <c r="C28" t="s">
-        <v>199</v>
-      </c>
-      <c r="D28" t="s">
-        <v>200</v>
-      </c>
-      <c r="E28" t="s">
-        <v>201</v>
-      </c>
-      <c r="F28" t="s">
-        <v>21</v>
-      </c>
-      <c r="G28" t="s">
-        <v>199</v>
-      </c>
-      <c r="H28" t="s">
-        <v>202</v>
-      </c>
-      <c r="I28" t="s">
-        <v>203</v>
-      </c>
-      <c r="J28" t="s">
-        <v>25</v>
-      </c>
-      <c r="K28" t="s">
-        <v>90</v>
-      </c>
-      <c r="L28" t="s">
-        <v>204</v>
-      </c>
-      <c r="M28" t="s">
-        <v>21</v>
-      </c>
-      <c r="N28" t="s">
-        <v>21</v>
-      </c>
-      <c r="O28" t="s">
-        <v>26</v>
-      </c>
-      <c r="P28" t="s">
-        <v>199</v>
-      </c>
-      <c r="Q28" t="s">
-        <v>199</v>
+      <c r="C29" t="s">
+        <v>250</v>
+      </c>
+      <c r="D29" t="s">
+        <v>251</v>
+      </c>
+      <c r="E29" t="s">
+        <v>252</v>
+      </c>
+      <c r="F29" t="s">
+        <v>28</v>
+      </c>
+      <c r="G29" t="s">
+        <v>250</v>
+      </c>
+      <c r="H29" t="s">
+        <v>253</v>
+      </c>
+      <c r="I29" t="s">
+        <v>254</v>
+      </c>
+      <c r="J29" t="s">
+        <v>32</v>
+      </c>
+      <c r="K29" t="s">
+        <v>107</v>
+      </c>
+      <c r="L29" t="s">
+        <v>255</v>
+      </c>
+      <c r="M29" t="s">
+        <v>28</v>
+      </c>
+      <c r="N29" t="s">
+        <v>28</v>
+      </c>
+      <c r="O29" t="s">
+        <v>250</v>
+      </c>
+      <c r="P29" t="s">
+        <v>250</v>
+      </c>
+      <c r="Q29" t="s">
+        <v>256</v>
+      </c>
+      <c r="R29" t="s">
+        <v>33</v>
+      </c>
+      <c r="S29" t="s">
+        <v>257</v>
+      </c>
+      <c r="T29" t="s">
+        <v>111</v>
+      </c>
+      <c r="U29" t="s">
+        <v>28</v>
+      </c>
+      <c r="V29" t="s">
+        <v>28</v>
+      </c>
+      <c r="W29" t="s">
+        <v>28</v>
+      </c>
+      <c r="X29" t="s">
+        <v>28</v>
       </c>
     </row>
-    <row r="29" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A29" t="s">
-        <v>205</v>
-      </c>
-      <c r="B29">
-        <v>1</v>
-      </c>
-      <c r="C29" t="s">
-        <v>206</v>
-      </c>
-      <c r="D29" t="s">
-        <v>207</v>
-      </c>
-      <c r="E29" t="s">
-        <v>208</v>
-      </c>
-      <c r="F29" t="s">
-        <v>21</v>
-      </c>
-      <c r="G29" t="s">
-        <v>206</v>
-      </c>
-      <c r="H29" t="s">
-        <v>209</v>
-      </c>
-      <c r="I29" t="s">
-        <v>210</v>
-      </c>
-      <c r="J29" t="s">
-        <v>25</v>
-      </c>
-      <c r="K29" t="s">
-        <v>90</v>
-      </c>
-      <c r="L29" t="s">
-        <v>211</v>
-      </c>
-      <c r="M29" t="s">
-        <v>21</v>
-      </c>
-      <c r="N29" t="s">
-        <v>21</v>
-      </c>
-      <c r="O29" t="s">
-        <v>34</v>
-      </c>
-      <c r="P29" t="s">
-        <v>206</v>
-      </c>
-      <c r="Q29" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="30" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>212</v>
+        <v>258</v>
       </c>
       <c r="B30">
         <v>1</v>
       </c>
       <c r="C30" t="s">
-        <v>213</v>
+        <v>259</v>
       </c>
       <c r="D30" t="s">
-        <v>214</v>
+        <v>260</v>
       </c>
       <c r="E30" t="s">
-        <v>215</v>
+        <v>261</v>
       </c>
       <c r="F30" t="s">
-        <v>216</v>
+        <v>28</v>
       </c>
       <c r="G30" t="s">
-        <v>213</v>
+        <v>259</v>
       </c>
       <c r="H30" t="s">
-        <v>217</v>
+        <v>262</v>
       </c>
       <c r="I30" t="s">
-        <v>218</v>
+        <v>263</v>
       </c>
       <c r="J30" t="s">
-        <v>25</v>
+        <v>32</v>
       </c>
       <c r="K30" t="s">
-        <v>219</v>
+        <v>107</v>
       </c>
       <c r="L30" t="s">
-        <v>219</v>
+        <v>264</v>
       </c>
       <c r="M30" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="N30" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="O30" t="s">
-        <v>34</v>
+        <v>259</v>
       </c>
       <c r="P30" t="s">
-        <v>213</v>
+        <v>259</v>
       </c>
       <c r="Q30" t="s">
-        <v>213</v>
+        <v>265</v>
+      </c>
+      <c r="R30" t="s">
+        <v>33</v>
+      </c>
+      <c r="S30" t="s">
+        <v>266</v>
+      </c>
+      <c r="T30" t="s">
+        <v>267</v>
+      </c>
+      <c r="U30" t="s">
+        <v>28</v>
+      </c>
+      <c r="V30" t="s">
+        <v>28</v>
+      </c>
+      <c r="W30" t="s">
+        <v>28</v>
+      </c>
+      <c r="X30" t="s">
+        <v>28</v>
       </c>
     </row>
-    <row r="31" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>220</v>
+        <v>268</v>
       </c>
       <c r="B31">
         <v>1</v>
       </c>
       <c r="C31" t="s">
-        <v>147</v>
+        <v>269</v>
       </c>
       <c r="D31" t="s">
-        <v>221</v>
+        <v>270</v>
       </c>
       <c r="E31" t="s">
-        <v>222</v>
+        <v>271</v>
       </c>
       <c r="F31" t="s">
-        <v>147</v>
+        <v>121</v>
       </c>
       <c r="G31" t="s">
-        <v>223</v>
+        <v>269</v>
       </c>
       <c r="H31" t="s">
-        <v>224</v>
+        <v>272</v>
       </c>
       <c r="I31" t="s">
-        <v>225</v>
+        <v>273</v>
       </c>
       <c r="J31" t="s">
-        <v>25</v>
+        <v>32</v>
       </c>
       <c r="K31" t="s">
-        <v>162</v>
+        <v>274</v>
       </c>
       <c r="L31" t="s">
-        <v>163</v>
+        <v>274</v>
       </c>
       <c r="M31" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="N31" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="O31" t="s">
-        <v>34</v>
+        <v>269</v>
       </c>
       <c r="P31" t="s">
-        <v>223</v>
+        <v>269</v>
       </c>
       <c r="Q31" t="s">
-        <v>147</v>
+        <v>275</v>
+      </c>
+      <c r="R31" t="s">
+        <v>33</v>
+      </c>
+      <c r="S31" t="s">
+        <v>276</v>
+      </c>
+      <c r="T31" t="s">
+        <v>28</v>
+      </c>
+      <c r="U31" t="s">
+        <v>28</v>
+      </c>
+      <c r="V31" t="s">
+        <v>28</v>
+      </c>
+      <c r="W31" t="s">
+        <v>28</v>
+      </c>
+      <c r="X31" t="s">
+        <v>28</v>
       </c>
     </row>
-    <row r="32" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>226</v>
+        <v>277</v>
       </c>
       <c r="B32">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C32" t="s">
-        <v>227</v>
+        <v>183</v>
       </c>
       <c r="D32" t="s">
-        <v>228</v>
+        <v>278</v>
       </c>
       <c r="E32" t="s">
-        <v>229</v>
+        <v>279</v>
       </c>
       <c r="F32" t="s">
-        <v>21</v>
+        <v>183</v>
       </c>
       <c r="G32" t="s">
-        <v>227</v>
+        <v>280</v>
       </c>
       <c r="H32" t="s">
-        <v>186</v>
+        <v>281</v>
       </c>
       <c r="I32" t="s">
-        <v>230</v>
+        <v>282</v>
       </c>
       <c r="J32" t="s">
-        <v>25</v>
+        <v>32</v>
       </c>
       <c r="K32" t="s">
-        <v>90</v>
+        <v>170</v>
       </c>
       <c r="L32" t="s">
-        <v>231</v>
+        <v>171</v>
       </c>
       <c r="M32" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="N32" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="O32" t="s">
-        <v>26</v>
+        <v>280</v>
       </c>
       <c r="P32" t="s">
-        <v>227</v>
+        <v>183</v>
       </c>
       <c r="Q32" t="s">
-        <v>227</v>
+        <v>283</v>
+      </c>
+      <c r="R32" t="s">
+        <v>33</v>
+      </c>
+      <c r="S32" t="s">
+        <v>284</v>
+      </c>
+      <c r="T32" t="s">
+        <v>28</v>
+      </c>
+      <c r="U32" t="s">
+        <v>28</v>
+      </c>
+      <c r="V32" t="s">
+        <v>218</v>
+      </c>
+      <c r="W32" t="s">
+        <v>285</v>
+      </c>
+      <c r="X32" t="s">
+        <v>28</v>
       </c>
     </row>
-    <row r="33" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>232</v>
+        <v>286</v>
       </c>
       <c r="B33">
         <v>2</v>
       </c>
       <c r="C33" t="s">
-        <v>233</v>
+        <v>287</v>
       </c>
       <c r="D33" t="s">
-        <v>234</v>
+        <v>288</v>
       </c>
       <c r="E33" t="s">
-        <v>235</v>
+        <v>289</v>
       </c>
       <c r="F33" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="G33" t="s">
-        <v>233</v>
+        <v>287</v>
       </c>
       <c r="H33" t="s">
-        <v>186</v>
+        <v>237</v>
       </c>
       <c r="I33" t="s">
-        <v>236</v>
+        <v>290</v>
       </c>
       <c r="J33" t="s">
-        <v>25</v>
+        <v>32</v>
       </c>
       <c r="K33" t="s">
-        <v>90</v>
+        <v>107</v>
       </c>
       <c r="L33" t="s">
-        <v>231</v>
+        <v>291</v>
       </c>
       <c r="M33" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="N33" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="O33" t="s">
-        <v>26</v>
+        <v>287</v>
       </c>
       <c r="P33" t="s">
-        <v>233</v>
+        <v>287</v>
       </c>
       <c r="Q33" t="s">
-        <v>233</v>
+        <v>292</v>
+      </c>
+      <c r="R33" t="s">
+        <v>33</v>
+      </c>
+      <c r="S33" t="s">
+        <v>293</v>
+      </c>
+      <c r="T33" t="s">
+        <v>28</v>
+      </c>
+      <c r="U33" t="s">
+        <v>28</v>
+      </c>
+      <c r="V33" t="s">
+        <v>28</v>
+      </c>
+      <c r="W33" t="s">
+        <v>28</v>
+      </c>
+      <c r="X33" t="s">
+        <v>294</v>
       </c>
     </row>
-    <row r="34" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
+        <v>295</v>
+      </c>
+      <c r="B34">
+        <v>2</v>
+      </c>
+      <c r="C34" t="s">
+        <v>296</v>
+      </c>
+      <c r="D34" t="s">
+        <v>297</v>
+      </c>
+      <c r="E34" t="s">
+        <v>298</v>
+      </c>
+      <c r="F34" t="s">
+        <v>28</v>
+      </c>
+      <c r="G34" t="s">
+        <v>296</v>
+      </c>
+      <c r="H34" t="s">
         <v>237</v>
       </c>
-      <c r="B34">
-        <v>1</v>
-      </c>
-      <c r="C34" t="s">
-        <v>238</v>
-      </c>
-      <c r="D34" t="s">
-        <v>239</v>
-      </c>
-      <c r="E34" t="s">
-        <v>240</v>
-      </c>
-      <c r="F34" t="s">
-        <v>21</v>
-      </c>
-      <c r="G34" t="s">
-        <v>238</v>
-      </c>
-      <c r="H34" t="s">
-        <v>241</v>
-      </c>
       <c r="I34" t="s">
-        <v>242</v>
+        <v>299</v>
       </c>
       <c r="J34" t="s">
-        <v>25</v>
+        <v>32</v>
       </c>
       <c r="K34" t="s">
-        <v>243</v>
+        <v>107</v>
       </c>
       <c r="L34" t="s">
-        <v>244</v>
+        <v>291</v>
       </c>
       <c r="M34" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="N34" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="O34" t="s">
-        <v>34</v>
+        <v>296</v>
       </c>
       <c r="P34" t="s">
-        <v>238</v>
+        <v>296</v>
       </c>
       <c r="Q34" t="s">
-        <v>238</v>
+        <v>300</v>
+      </c>
+      <c r="R34" t="s">
+        <v>33</v>
+      </c>
+      <c r="S34" t="s">
+        <v>301</v>
+      </c>
+      <c r="T34" t="s">
+        <v>111</v>
+      </c>
+      <c r="U34" t="s">
+        <v>28</v>
+      </c>
+      <c r="V34" t="s">
+        <v>28</v>
+      </c>
+      <c r="W34" t="s">
+        <v>28</v>
+      </c>
+      <c r="X34" t="s">
+        <v>294</v>
       </c>
     </row>
-    <row r="35" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>245</v>
+        <v>302</v>
       </c>
       <c r="B35">
         <v>1</v>
       </c>
       <c r="C35" t="s">
-        <v>246</v>
+        <v>303</v>
       </c>
       <c r="D35" t="s">
-        <v>247</v>
+        <v>304</v>
       </c>
       <c r="E35" t="s">
-        <v>248</v>
+        <v>305</v>
       </c>
       <c r="F35" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="G35" t="s">
-        <v>249</v>
+        <v>303</v>
       </c>
       <c r="H35" t="s">
-        <v>250</v>
+        <v>306</v>
       </c>
       <c r="I35" t="s">
-        <v>251</v>
+        <v>307</v>
       </c>
       <c r="J35" t="s">
-        <v>25</v>
+        <v>32</v>
       </c>
       <c r="K35" t="s">
-        <v>21</v>
+        <v>308</v>
       </c>
       <c r="L35" t="s">
-        <v>21</v>
+        <v>309</v>
       </c>
       <c r="M35" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="N35" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="O35" t="s">
-        <v>26</v>
+        <v>303</v>
       </c>
       <c r="P35" t="s">
-        <v>246</v>
+        <v>303</v>
       </c>
       <c r="Q35" t="s">
-        <v>246</v>
+        <v>310</v>
+      </c>
+      <c r="R35" t="s">
+        <v>33</v>
+      </c>
+      <c r="S35" t="s">
+        <v>311</v>
+      </c>
+      <c r="T35" t="s">
+        <v>28</v>
+      </c>
+      <c r="U35" t="s">
+        <v>28</v>
+      </c>
+      <c r="V35" t="s">
+        <v>28</v>
+      </c>
+      <c r="W35" t="s">
+        <v>28</v>
+      </c>
+      <c r="X35" t="s">
+        <v>28</v>
       </c>
     </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>21</v>
+        <v>312</v>
+      </c>
+      <c r="B36">
+        <v>1</v>
+      </c>
+      <c r="C36" t="s">
+        <v>313</v>
+      </c>
+      <c r="D36" t="s">
+        <v>314</v>
+      </c>
+      <c r="E36" t="s">
+        <v>315</v>
+      </c>
+      <c r="F36" t="s">
+        <v>28</v>
+      </c>
+      <c r="G36" t="s">
+        <v>316</v>
+      </c>
+      <c r="H36" t="s">
+        <v>317</v>
+      </c>
+      <c r="I36" t="s">
+        <v>318</v>
+      </c>
+      <c r="J36" t="s">
+        <v>32</v>
+      </c>
+      <c r="K36" t="s">
+        <v>28</v>
+      </c>
+      <c r="L36" t="s">
+        <v>28</v>
+      </c>
+      <c r="M36" t="s">
+        <v>28</v>
+      </c>
+      <c r="N36" t="s">
+        <v>28</v>
+      </c>
+      <c r="O36" t="s">
+        <v>313</v>
+      </c>
+      <c r="P36" t="s">
+        <v>313</v>
+      </c>
+      <c r="Q36" t="s">
+        <v>28</v>
+      </c>
+      <c r="R36" t="s">
+        <v>33</v>
+      </c>
+      <c r="S36" t="s">
+        <v>28</v>
+      </c>
+      <c r="T36" t="s">
+        <v>28</v>
+      </c>
+      <c r="U36" t="s">
+        <v>28</v>
+      </c>
+      <c r="V36" t="s">
+        <v>28</v>
+      </c>
+      <c r="W36" t="s">
+        <v>28</v>
+      </c>
+      <c r="X36" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="37" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>28</v>
       </c>
     </row>
   </sheetData>

</xml_diff>